<commit_message>
Finished Excel integration and UI updates
</commit_message>
<xml_diff>
--- a/ClinicVetsData.xlsx
+++ b/ClinicVetsData.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <x:workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\royal\source\repos\ClinicVets\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{BB042FC4-6CFC-4336-A45C-B28A4884A8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{9C3D8762-7773-4936-BFF2-DD921C98C03C}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Customer" sheetId="1" r:id="rId1"/>
-    <sheet name="Pets" sheetId="2" r:id="rId2"/>
-    <sheet name="Employees" sheetId="3" r:id="rId3"/>
-    <sheet name="Visits" sheetId="4" r:id="rId4"/>
-    <sheet name="Medicines" sheetId="5" r:id="rId5"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <x:bookViews>
+    <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{9C3D8762-7773-4936-BFF2-DD921C98C03C}"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet name="Customer" sheetId="1" r:id="rId1"/>
+    <x:sheet name="Pets" sheetId="2" r:id="rId2"/>
+    <x:sheet name="Employees" sheetId="3" r:id="rId3"/>
+    <x:sheet name="Visits" sheetId="4" r:id="rId4"/>
+    <x:sheet name="Medicines" sheetId="5" r:id="rId5"/>
+  </x:sheets>
+  <x:calcPr calcId="191029"/>
+  <x:extLst>
+    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+    </x:ext>
+    <x:ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
@@ -34,107 +34,107 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+    </x:ext>
+    <x:ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
-</workbook>
+    </x:ext>
+  </x:extLst>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
-  <si>
-    <t>CustomerID</t>
-  </si>
-  <si>
-    <t>FullName</t>
-  </si>
-  <si>
-    <t>IDNumber</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>PetID</t>
-  </si>
-  <si>
-    <t>PetName</t>
-  </si>
-  <si>
-    <t>AnimalType</t>
-  </si>
-  <si>
-    <t>Weight</t>
-  </si>
-  <si>
-    <t>BirthDate</t>
-  </si>
-  <si>
-    <t>ChipNumber</t>
-  </si>
-  <si>
-    <t>OwnerID</t>
-  </si>
-  <si>
-    <t>LastVaccineDate</t>
-  </si>
-  <si>
-    <t>EmployeeID</t>
-  </si>
-  <si>
-    <t>Username</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>NationalID</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>VisitID</t>
-  </si>
-  <si>
-    <t>VisitDate</t>
-  </si>
-  <si>
-    <t>VisitTime</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>Diagnosis</t>
-  </si>
-  <si>
-    <t>Medicines</t>
-  </si>
-  <si>
-    <t>VetName</t>
-  </si>
-  <si>
-    <t>TotalPrice</t>
-  </si>
-  <si>
-    <t>MedicineID</t>
-  </si>
-  <si>
-    <t>MedicineName</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>StockQuantity</t>
-  </si>
-</sst>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+  <x:si>
+    <x:t>CustomerID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FullName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IDNumber</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Phone</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Email</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PetID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PetName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AnimalType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BirthDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ChipNumber</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OwnerID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LastVaccineDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EmployeeID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Username</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Password</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NationalID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Role</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VisitID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VisitDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VisitTime</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Reason</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Diagnosis</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Medicines</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VetName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TotalPrice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MedicineID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MedicineName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Price</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StockQuantity</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -503,36 +503,63 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C29998A4-787D-4E4F-8880-F98F419ED5E1}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.59765625" customWidth="1"/>
-    <col min="2" max="2" width="11.59765625" customWidth="1"/>
-    <col min="3" max="4" width="12.3984375" customWidth="1"/>
-    <col min="5" max="5" width="12.09765625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{C29998A4-787D-4E4F-8880-F98F419ED5E1}" mc:Ignorable="x14ac xr xr2 xr3">
+  <x:dimension ref="A1:E1"/>
+  <x:sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14.59765625" customWidth="1"/>
+    <x:col min="2" max="2" width="11.59765625" customWidth="1"/>
+    <x:col min="3" max="4" width="12.3984375" customWidth="1"/>
+    <x:col min="5" max="5" width="12.09765625" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <x:c r="A1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="inlineStr">
+        <x:is>
+          <x:t>trrrrrry@gmail.com</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" t="inlineStr">
+        <x:is>
+          <x:t>0502573118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" t="inlineStr">
+        <x:is>
+          <x:t>325698741</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" t="inlineStr">
+        <x:is>
+          <x:t>ssssso</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" t="inlineStr">
+        <x:is>
+          <x:t>147808635c9243c5887269207400e059</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update pets Excel logic
</commit_message>
<xml_diff>
--- a/ClinicVetsData.xlsx
+++ b/ClinicVetsData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\royal\source\repos\ClinicVets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB042FC4-6CFC-4336-A45C-B28A4884A8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1A7F9E-FD0C-4A43-B4E9-ACC68BC78901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
-    <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="0" activeTab="4" xr2:uid="{9C3D8762-7773-4936-BFF2-DD921C98C03C}"/>
+    <x:workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="0" activeTab="1" xr2:uid="{9C3D8762-7773-4936-BFF2-DD921C98C03C}"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <x:sheet name="Employees" sheetId="3" r:id="rId3"/>
     <x:sheet name="Visits" sheetId="4" r:id="rId4"/>
     <x:sheet name="Medicines" sheetId="5" r:id="rId5"/>
+    <x:sheet name="AnimalTypes" sheetId="6" r:id="rId6"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="191029"/>
@@ -61,28 +62,40 @@
     <x:t>CustomerID</x:t>
   </x:si>
   <x:si>
+    <x:t>PetID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PetName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AnimalType</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BirthDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ChipNumber</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OwnerID</x:t>
+  </x:si>
+  <x:si>
     <x:t>LastVaccineDate</x:t>
   </x:si>
   <x:si>
-    <x:t>OwnerID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ChipNumber</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BirthDate</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weight</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AnimalType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PetName</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PetID</x:t>
+    <x:t>P001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>max</x:t>
+  </x:si>
+  <x:si>
+    <x:t>avi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>001</x:t>
   </x:si>
   <x:si>
     <x:t>Role</x:t>
@@ -140,6 +153,18 @@
   </x:si>
   <x:si>
     <x:t>acamols</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AnimalTypes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Dog</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Reptile</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -182,11 +207,15 @@
       <x:diagonal/>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,7 +592,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H1"/>
+  <x:dimension ref="A1:H2"/>
   <x:sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <x:cols>
     <x:col min="1" max="1" width="15.898438" style="0" customWidth="1"/>
@@ -572,7 +601,7 @@
     <x:col min="4" max="4" width="10.699219" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.5" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="12.699219" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="9.090625" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.097656" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="11.199219" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -600,6 +629,32 @@
       </x:c>
       <x:c r="H1" s="0" t="s">
         <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="D2" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E2" s="1">
+        <x:v>46149</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H2" s="1">
+        <x:v>46156</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -621,7 +676,7 @@
   <x:cols>
     <x:col min="1" max="1" width="11" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="10.898438" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9.090625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.097656" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="11.398438" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="12.199219" style="0" customWidth="1"/>
@@ -629,22 +684,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -677,31 +732,31 @@
   <x:sheetData>
     <x:row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -718,30 +773,30 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D1"/>
+  <x:dimension ref="A1:D3"/>
   <x:sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.585625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.085625" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13.460625" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.460625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.597656" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.097656" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.5" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.5" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:4">
+        <x:v>33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <x:c r="A2" s="0">
         <x:v>321</x:v>
       </x:c>
@@ -749,13 +804,13 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:4">
+    <x:row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <x:c r="A3" s="0">
         <x:v>144</x:v>
       </x:c>
@@ -763,10 +818,50 @@
         <x:v>1234</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{36630A44-FD62-4C72-8549-8361A9DCCCD8}" mc:Ignorable="x14ac xr xr2 xr3">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:A4"/>
+  <x:sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13.398438" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A1" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A2" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A3" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <x:c r="A4" s="0" t="s">
+        <x:v>39</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
backup before performance cleanup
</commit_message>
<xml_diff>
--- a/ClinicVetsData.xlsx
+++ b/ClinicVetsData.xlsx
@@ -686,9 +686,6 @@
       <x:c r="A1" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -698,8 +695,14 @@
       <x:c r="E1" s="0" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="F1" s="0" t="s">
-        <x:v>21</x:v>
+      <x:c r="F1" t="str">
+        <x:v>EmployeeNumber</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>FullName</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>NationalID</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -796,6 +799,144 @@
         <x:is>
           <x:t>Secretary</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="F5" t="str">
+        <x:v>8881</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>ccccbg</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>ghgG5!d</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>jwhj@gmail.com</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>326011587</x:v>
+      </x:c>
+      <x:c r="A5" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>dgher</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="F6" t="str">
+        <x:v>8585</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>ppipg11</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>gmei</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>ffF7F7!</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>dgaG@gmail.com</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>852369977</x:v>
+      </x:c>
+      <x:c r="A6" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>987456321</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>hsg@gmail.com</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>fgdH45!</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>sjgkdg</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>7899</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>rtsyhsh</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>852852852</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>vdg@gmail.com</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>jhJ5851!</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>ihggkl</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>1115</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>vhgjhg</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>852852852</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>gsfd@gmail.com</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>dfbH78!</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>kjdgfn</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>8853</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>dsisn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Vet</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>747185296</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>jolana@gmail.com</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Julana1!</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Jhamm</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>7417</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>julana</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Fix UI and clinic workflow updates
</commit_message>
<xml_diff>
--- a/ClinicVetsData.xlsx
+++ b/ClinicVetsData.xlsx
@@ -62,6 +62,18 @@
     <x:t>CustomerID</x:t>
   </x:si>
   <x:si>
+    <x:t>sdfdf@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0523164978</x:t>
+  </x:si>
+  <x:si>
+    <x:t>123456989</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lameaa</x:t>
+  </x:si>
+  <x:si>
     <x:t>PetID</x:t>
   </x:si>
   <x:si>
@@ -92,12 +104,33 @@
     <x:t>max</x:t>
   </x:si>
   <x:si>
+    <x:t>Dog</x:t>
+  </x:si>
+  <x:si>
     <x:t>avi</x:t>
   </x:si>
   <x:si>
     <x:t>001</x:t>
   </x:si>
   <x:si>
+    <x:t>coroo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lolo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fofo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Role</x:t>
   </x:si>
   <x:si>
@@ -110,7 +143,154 @@
     <x:t>Username</x:t>
   </x:si>
   <x:si>
-    <x:t>EmployeeID</x:t>
+    <x:t>EmployeeNumber</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vet</x:t>
+  </x:si>
+  <x:si>
+    <x:t>326011587</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jwhj@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ghgG5!d</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ccccbg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8881</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dgher</x:t>
+  </x:si>
+  <x:si>
+    <x:t>852369977</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dgaG@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ffF7F7!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ppipg11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8585</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gmei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>987456321</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hsg@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fgdH45!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sjgkdg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7899</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rtsyhsh</x:t>
+  </x:si>
+  <x:si>
+    <x:t>852852852</x:t>
+  </x:si>
+  <x:si>
+    <x:t>vdg@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jhJ5851!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ihggkl</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1115</x:t>
+  </x:si>
+  <x:si>
+    <x:t>vhgjhg</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gsfd@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dfbH78!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kjdgfn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8853</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dsisn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>747185296</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jolana@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Julana12!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jhamm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7417</x:t>
+  </x:si>
+  <x:si>
+    <x:t>julana</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Secretary</x:t>
+  </x:si>
+  <x:si>
+    <x:t>123123127</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ujghf@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jul111!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sharonn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8527</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sharo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>789654123</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gdfg@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kal111!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fathia</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0009</x:t>
+  </x:si>
+  <x:si>
+    <x:t>julana elelqamawi</x:t>
   </x:si>
   <x:si>
     <x:t>TotalPrice</x:t>
@@ -137,6 +317,117 @@
     <x:t>VisitID</x:t>
   </x:si>
   <x:si>
+    <x:t>P001 — coroo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25/05/2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04:25 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>nos pain</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>1234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jhamm</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100 NIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P001 — max</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04:42 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>pain</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:20 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>njdfj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:29 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fds</x:t>
+  </x:si>
+  <x:si>
+    <x:t>afeqr</x:t>
+  </x:si>
+  <x:si>
+    <x:t>200 NIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:33 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jhgkug kjbh</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:53 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pain ijfh </x:t>
+  </x:si>
+  <x:si>
+    <x:t>1334 NIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:54 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>p;jhj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>uhbk,</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05:55 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rfghj</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gujhkn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100, 1234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1434 NIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06:04 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ogkp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mynrbtgrfv</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06:05 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>nkk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ilkn,m</x:t>
+  </x:si>
+  <x:si>
     <x:t>StockQuantity</x:t>
   </x:si>
   <x:si>
@@ -149,22 +440,37 @@
     <x:t>MedicineID</x:t>
   </x:si>
   <x:si>
+    <x:t>Status</x:t>
+  </x:si>
+  <x:si>
     <x:t>acamol</x:t>
   </x:si>
   <x:si>
     <x:t>acamols</x:t>
   </x:si>
   <x:si>
+    <x:t>advil</x:t>
+  </x:si>
+  <x:si>
+    <x:t>panadol</x:t>
+  </x:si>
+  <x:si>
     <x:t>AnimalTypes</x:t>
   </x:si>
   <x:si>
-    <x:t>Dog</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cat</x:t>
-  </x:si>
-  <x:si>
     <x:t>Reptile</x:t>
+  </x:si>
+  <x:si>
+    <x:t>06:19 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sdfghjk</x:t>
+  </x:si>
+  <x:si>
+    <x:t>tyuhiko dfghjk i</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Available</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -578,6 +884,23 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -607,39 +930,39 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <x:c r="A2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>7</x:v>
@@ -648,13 +971,65 @@
         <x:v>46149</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H2" s="1">
         <x:v>46156</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8">
+      <x:c r="A3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E3" s="1">
+        <x:v>46030</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H3" s="1">
+        <x:v>46167</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:8">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="1">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="H4" s="1">
+        <x:v>46167</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -682,261 +1057,307 @@
     <x:col min="6" max="6" width="12.199219" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <x:row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F1" t="str">
-        <x:v>EmployeeNumber</x:v>
-      </x:c>
-      <x:c r="G1" t="str">
-        <x:v>FullName</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>NationalID</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="E2" t="inlineStr">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="inlineStr">
+        <x:is>
+          <x:t>Vet</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="0" t="inlineStr">
+        <x:is>
+          <x:t>326011585</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="0" t="inlineStr">
+        <x:is>
+          <x:t>julana137@gmail.com</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="0" t="inlineStr">
+        <x:is>
+          <x:t>Julana1!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="0" t="inlineStr">
         <x:is>
           <x:t>julana</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t>Julana1!</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F2" t="inlineStr">
+      <x:c r="F2" s="0" t="inlineStr">
         <x:is>
           <x:t>1265</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" t="inlineStr">
+    </x:row>
+    <x:row r="3" spans="1:7">
+      <x:c r="A3" s="0" t="inlineStr">
         <x:is>
-          <x:t>julana137@gmail.com</x:t>
+          <x:t>Secretary</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" t="inlineStr">
+      <x:c r="B3" s="0" t="inlineStr">
         <x:is>
-          <x:t>326011585</x:t>
+          <x:t>326598747</x:t>
         </x:is>
       </x:c>
-      <x:c r="A2" t="inlineStr">
+      <x:c r="C3" s="0" t="inlineStr">
         <x:is>
-          <x:t>Vet</x:t>
+          <x:t>sharon@gmail.com</x:t>
         </x:is>
       </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="E3" t="inlineStr">
+      <x:c r="D3" s="0" t="inlineStr">
+        <x:is>
+          <x:t>Sharo1!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="0" t="inlineStr">
         <x:is>
           <x:t>sharon</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t>Sharo1!</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" t="inlineStr">
+      <x:c r="F3" s="0" t="inlineStr">
         <x:is>
           <x:t>7891</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t>sharon@gmail.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t>326598747</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="A3" t="inlineStr">
+    </x:row>
+    <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="inlineStr">
         <x:is>
           <x:t>Secretary</x:t>
         </x:is>
       </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="E4" t="inlineStr">
+      <x:c r="B4" s="0" t="inlineStr">
+        <x:is>
+          <x:t>326512326</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="0" t="inlineStr">
+        <x:is>
+          <x:t>elelqamawi.sharon@gmail.com</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="0" t="inlineStr">
+        <x:is>
+          <x:t>shAron1!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="0" t="inlineStr">
         <x:is>
           <x:t>sharoo</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" t="inlineStr">
-        <x:is>
-          <x:t>shAron1!</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" t="inlineStr">
+      <x:c r="F4" s="0" t="inlineStr">
         <x:is>
           <x:t>1231</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t>elelqamawi.sharon@gmail.com</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t>326512326</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t>Secretary</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="F5" t="str">
-        <x:v>8881</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>ccccbg</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
-        <x:v>ghgG5!d</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>jwhj@gmail.com</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>326011587</x:v>
-      </x:c>
-      <x:c r="A5" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-      <x:c r="G5" t="str">
-        <x:v>dgher</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="F6" t="str">
-        <x:v>8585</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>ppipg11</x:v>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:v>gmei</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
-        <x:v>ffF7F7!</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>dgaG@gmail.com</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>852369977</x:v>
-      </x:c>
-      <x:c r="A6" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>987456321</x:v>
-      </x:c>
-      <x:c r="C7" t="str">
-        <x:v>hsg@gmail.com</x:v>
-      </x:c>
-      <x:c r="D7" t="str">
-        <x:v>fgdH45!</x:v>
-      </x:c>
-      <x:c r="E7" t="str">
-        <x:v>sjgkdg</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>7899</x:v>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:v>rtsyhsh</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>852852852</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>vdg@gmail.com</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>jhJ5851!</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>ihggkl</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>1115</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>vhgjhg</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>852852852</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>gsfd@gmail.com</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>dfbH78!</x:v>
-      </x:c>
-      <x:c r="E9" t="str">
-        <x:v>kjdgfn</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>8853</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>dsisn</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Vet</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>747185296</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>jolana@gmail.com</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>Julana1!</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>Jhamm</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>7417</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>julana</x:v>
+    </x:row>
+    <x:row r="5" spans="1:7">
+      <x:c r="A5" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="A7" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="A9" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
+      <x:c r="A11" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:7">
+      <x:c r="A12" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="F12" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="G12" s="0" t="s">
+        <x:v>81</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -969,31 +1390,350 @@
   <x:sheetData>
     <x:row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:9">
+      <x:c r="A2" s="0">
+        <x:v>6741</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:9">
+      <x:c r="A3" s="0">
+        <x:v>8595</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:9">
+      <x:c r="A4" s="0">
+        <x:v>3417</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:9">
+      <x:c r="A5" s="0">
+        <x:v>2762</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:9">
+      <x:c r="A6" s="0">
+        <x:v>3654</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:9">
+      <x:c r="A7" s="0">
+        <x:v>6627</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="I7" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:9">
+      <x:c r="A8" s="0">
+        <x:v>9311</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I8" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:9">
+      <x:c r="A9" s="0">
+        <x:v>4033</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="I9" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:9">
+      <x:c r="A10" s="0">
+        <x:v>7073</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H10" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="I10" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:9">
+      <x:c r="A11" s="0">
+        <x:v>9632</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H11" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="I11" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:9">
+      <x:c r="A12" s="0">
+        <x:v>1795</x:v>
+      </x:c>
+      <x:c r="B12" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="F12" s="0" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="G12" s="0" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="H12" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="I12" s="0" t="s">
+        <x:v>112</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1013,52 +1753,86 @@
   <x:dimension ref="A1:D3"/>
   <x:sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.597656" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.097656" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13.5" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10.5" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.585625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.085625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.460625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.460625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <x:row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>131</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <x:c r="A2" s="0">
-        <x:v>321</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>100</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <x:row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <x:c r="A3" s="0">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B3" s="0">
         <x:v>1234</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>2</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>141</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="0">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1083,22 +1857,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A2" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A4" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Fix pet validation and complete navigation flow
</commit_message>
<xml_diff>
--- a/ClinicVetsData.xlsx
+++ b/ClinicVetsData.xlsx
@@ -108,6 +108,51 @@
     <x:t>6</x:t>
   </x:si>
   <x:si>
+    <x:t>aaa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>bird</x:t>
+  </x:si>
+  <x:si>
+    <x:t>012</x:t>
+  </x:si>
+  <x:si>
+    <x:t>raji</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lol</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Reptile</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0009</x:t>
+  </x:si>
+  <x:si>
+    <x:t>pop</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fofo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0019</x:t>
+  </x:si>
+  <x:si>
+    <x:t>popo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1113</x:t>
+  </x:si>
+  <x:si>
     <x:t>Role</x:t>
   </x:si>
   <x:si>
@@ -306,6 +351,24 @@
     <x:t>4512</x:t>
   </x:si>
   <x:si>
+    <x:t>326011579</x:t>
+  </x:si>
+  <x:si>
+    <x:t>julana.elsayed137@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Julana13!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>julana07</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0017</x:t>
+  </x:si>
+  <x:si>
+    <x:t>julana elelqamawi</x:t>
+  </x:si>
+  <x:si>
     <x:t>TotalPrice</x:t>
   </x:si>
   <x:si>
@@ -381,19 +444,10 @@
     <x:t>AnimalTypes</x:t>
   </x:si>
   <x:si>
-    <x:t>Cat</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Reptile</x:t>
-  </x:si>
-  <x:si>
-    <x:t>bird</x:t>
-  </x:si>
-  <x:si>
-    <x:t>aaa</x:t>
-  </x:si>
-  <x:si>
-    <x:t>012</x:t>
+    <x:t>gai</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0055</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -948,10 +1002,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="0">
         <x:v>4</x:v>
@@ -963,10 +1017,166 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H4" s="1">
         <x:v>46161</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:8">
+      <x:c r="A5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E5" s="1">
+        <x:v>46058</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H5" s="1">
+        <x:v>46121</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:8">
+      <x:c r="A6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D6" s="0">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E6" s="1">
+        <x:v>46143</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="H6" s="1">
+        <x:v>46160</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:8">
+      <x:c r="A7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D7" s="0">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E7" s="1">
+        <x:v>46143</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="H7" s="1">
+        <x:v>46166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:8">
+      <x:c r="A8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D8" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E8" s="1">
+        <x:v>46173</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="H8" s="1">
+        <x:v>46173</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:8">
+      <x:c r="A9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D9" s="0">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E9" s="1">
+        <x:v>46173</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H9" s="1">
+        <x:v>46150</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:8">
+      <x:c r="A10" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D10" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E10" s="1">
+        <x:v>46145</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="H10" s="1">
+        <x:v>46159</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -996,22 +1206,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
         <x:v>3</x:v>
@@ -1019,246 +1229,269 @@
     </x:row>
     <x:row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A2" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A3" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A4" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A5" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A6" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A7" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A8" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A9" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="G9" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A10" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <x:c r="A11" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="G11" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:7">
       <x:c r="A12" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>99</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:7">
+      <x:c r="A13" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="F13" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="G13" s="0" t="s">
+        <x:v>110</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1294,31 +1527,31 @@
   <x:sheetData>
     <x:row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9">
@@ -1326,28 +1559,28 @@
         <x:v>8809</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="H2" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -1355,28 +1588,28 @@
         <x:v>4222</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1404,16 +1637,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1424,7 +1657,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>1</x:v>
@@ -1438,7 +1671,7 @@
         <x:v>1234</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>2</x:v>
@@ -1466,7 +1699,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A1" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1476,17 +1709,17 @@
     </x:row>
     <x:row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A3" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A4" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <x:c r="A5" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>